<commit_message>
feat(core): Phase 2 & 3 Agentic Upgrade - PDCA loop, Gemini integration, Knapsack algorithm, Cloud Run Docker, CI/CD Actions
</commit_message>
<xml_diff>
--- a/CIRO_Emergencies_contact_details_UPDATED_FORMATTED.xlsx
+++ b/CIRO_Emergencies_contact_details_UPDATED_FORMATTED.xlsx
@@ -932,22 +932,22 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1020</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+92-21-99201300</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1700</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1700</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -1398,12 +1398,12 @@
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1700</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1700</t>
         </is>
       </c>
     </row>
@@ -1593,12 +1593,12 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1700</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1700</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -1608,12 +1608,12 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1700</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1700</t>
         </is>
       </c>
     </row>
@@ -1816,12 +1816,12 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+92-51-9271000</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+92-51-9271000</t>
         </is>
       </c>
       <c r="E36" s="14" t="inlineStr">
@@ -1831,12 +1831,12 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+92-51-9271000</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+92-51-9271000</t>
         </is>
       </c>
     </row>
@@ -1921,12 +1921,12 @@
       </c>
       <c r="C39" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1991</t>
         </is>
       </c>
       <c r="D39" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1991</t>
         </is>
       </c>
       <c r="E39" s="26" t="inlineStr">
@@ -1936,12 +1936,12 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1991</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1991</t>
         </is>
       </c>
     </row>
@@ -2371,12 +2371,12 @@
       </c>
       <c r="C53" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0317-4288665</t>
         </is>
       </c>
       <c r="D53" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0317-4288665</t>
         </is>
       </c>
       <c r="E53" s="36" t="inlineStr">
@@ -2386,12 +2386,12 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0317-4288665</t>
         </is>
       </c>
       <c r="G53" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0317-4288665</t>
         </is>
       </c>
     </row>
@@ -2511,12 +2511,12 @@
       </c>
       <c r="C57" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0800-01234</t>
         </is>
       </c>
       <c r="D57" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0800-01234</t>
         </is>
       </c>
       <c r="E57" s="36" t="inlineStr">
@@ -2526,12 +2526,12 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0800-01234</t>
         </is>
       </c>
       <c r="G57" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0800-01234</t>
         </is>
       </c>
     </row>

</xml_diff>